<commit_message>
Integration Stufe II Teil 2: Glue WS-G/WS-A2
- vofi_stubs(): vofi_mc, vofi_compare, vofi_sensitivity, vofi_solve (WS-G) und
  vofi_excel_template (WS-A2) gestrichen; Huelle in helper-ws-g.R entfernt
- test-scenario-read: Excel-Lesen/-Schreiben ist geliefert (Hinweise WS-A2)
- test-oracles: Vergleichskennzahlen (12.6) sind keine Registry-Kennzahlen und
  fuehren nicht mehr zum Skip; prob_better_than_ref von Orakel (g) wird jetzt
  ueber vofi_compare() geprueft
- Batch-Test 11 (Entscheidungsknoten: Kompositum = getrennte Rechnung) mit dem
  Foerder-Expander von WS-E2 ergaenzt statt unbedingtem Skip
- roxygenise: print.vofi_solution (NAMESPACE, man/), Doku WS-G/WS-A2
- Excel-Vorlage mit den Typen von WS-E2 (grant, tax_credit_35c) neu erzeugt;
  JSON-Schema war bereits aktuell

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WsrG8LieorBE65SqpGzj3D
</commit_message>
<xml_diff>
--- a/inst/templates/vofi_eingabe.xlsx
+++ b/inst/templates/vofi_eingabe.xlsx
@@ -4132,7 +4132,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2313" uniqueCount="2313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2316" uniqueCount="2316">
   <si>
     <t xml:space="preserve">VoFi-Eingabevorlage (Vollständiger Finanzplan mit Monte-Carlo-Simulation)</t>
   </si>
@@ -10716,6 +10716,9 @@
     <t xml:space="preserve">share_of</t>
   </si>
   <si>
+    <t xml:space="preserve">tax_credit_35c</t>
+  </si>
+  <si>
     <t xml:space="preserve">tenant_costs</t>
   </si>
   <si>
@@ -10734,6 +10737,9 @@
     <t xml:space="preserve">Energiekosten eines Segments</t>
   </si>
   <si>
+    <t xml:space="preserve">Investitionszuschuss</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ersparte Miete</t>
   </si>
   <si>
@@ -10756,6 +10762,9 @@
   </si>
   <si>
     <t xml:space="preserve">Anteil an anderen Zeilen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steuerermäßigung § 35c EStG</t>
   </si>
   <si>
     <t xml:space="preserve">Heizkosten der Mieter</t>
@@ -12573,7 +12582,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0">
           <x14:formula1>
-            <xm:f>'Listen'!$EX$3:$EX$20</xm:f>
+            <xm:f>'Listen'!$EX$3:$EX$22</xm:f>
           </x14:formula1>
           <xm:sqref>B3:B52</xm:sqref>
         </x14:dataValidation>
@@ -22309,25 +22318,25 @@
         <v>2179</v>
       </c>
       <c r="EX3" s="4" t="s">
-        <v>2195</v>
+        <v>2196</v>
       </c>
       <c r="EY3" s="4" t="s">
-        <v>2209</v>
+        <v>2212</v>
       </c>
       <c r="EZ3" s="4" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="FA3" s="4" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="FB3" s="4" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="FC3" s="4" t="s">
         <v>1995</v>
       </c>
       <c r="FD3" s="4" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
     </row>
     <row r="4">
@@ -22791,25 +22800,25 @@
         <v>2180</v>
       </c>
       <c r="EX4" s="4" t="s">
-        <v>2196</v>
+        <v>2197</v>
       </c>
       <c r="EY4" s="4" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="EZ4" s="4" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="FA4" s="4" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="FB4" s="4" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="FC4" s="4" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="FD4" s="4" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="5">
@@ -23145,25 +23154,25 @@
         <v>2181</v>
       </c>
       <c r="EX5" s="4" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
       <c r="EY5" s="4" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="EZ5" s="4" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="FA5" s="4" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="FB5" s="4" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="FC5" s="4" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="FD5" s="4" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="6">
@@ -23439,25 +23448,25 @@
         <v>2182</v>
       </c>
       <c r="EX6" s="4" t="s">
-        <v>2198</v>
+        <v>2199</v>
       </c>
       <c r="EY6" s="4" t="s">
-        <v>2212</v>
+        <v>2215</v>
       </c>
       <c r="EZ6" s="4" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="FA6" s="4" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="FB6" s="4" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="FC6" s="4" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="FD6" s="4" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="7">
@@ -23701,25 +23710,25 @@
         <v>2183</v>
       </c>
       <c r="EX7" s="4" t="s">
-        <v>2199</v>
+        <v>2200</v>
       </c>
       <c r="EY7" s="4" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="EZ7" s="4" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="FA7" s="4" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="FB7" s="4" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="FC7" s="4" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="FD7" s="4" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="8">
@@ -23946,22 +23955,22 @@
         <v>2177</v>
       </c>
       <c r="EY8" s="4" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="EZ8" s="4" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="FA8" s="4" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="FB8" s="4" t="s">
-        <v>2202</v>
+        <v>2204</v>
       </c>
       <c r="FC8" s="4" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="FD8" s="4" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="9">
@@ -24162,28 +24171,28 @@
       <c r="EU9" s="4"/>
       <c r="EV9" s="4"/>
       <c r="EW9" s="4" t="s">
-        <v>2184</v>
+        <v>1876</v>
       </c>
       <c r="EX9" s="4" t="s">
-        <v>2200</v>
+        <v>2201</v>
       </c>
       <c r="EY9" s="4" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="EZ9" s="4" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="FA9" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="FB9" s="4" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="FC9" s="4" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="FD9" s="4" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
     </row>
     <row r="10">
@@ -24376,24 +24385,24 @@
       <c r="EU10" s="4"/>
       <c r="EV10" s="4"/>
       <c r="EW10" s="4" t="s">
-        <v>2185</v>
+        <v>2184</v>
       </c>
       <c r="EX10" s="4" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="EY10" s="4" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="EZ10" s="4" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="FA10" s="4"/>
       <c r="FB10" s="4"/>
       <c r="FC10" s="4" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="FD10" s="4" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="11">
@@ -24582,20 +24591,20 @@
       <c r="EU11" s="4"/>
       <c r="EV11" s="4"/>
       <c r="EW11" s="4" t="s">
-        <v>2186</v>
+        <v>2185</v>
       </c>
       <c r="EX11" s="4" t="s">
-        <v>717</v>
+        <v>2203</v>
       </c>
       <c r="EY11" s="4"/>
       <c r="EZ11" s="4"/>
       <c r="FA11" s="4"/>
       <c r="FB11" s="4"/>
       <c r="FC11" s="4" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="FD11" s="4" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="12">
@@ -24772,20 +24781,20 @@
       <c r="EU12" s="4"/>
       <c r="EV12" s="4"/>
       <c r="EW12" s="4" t="s">
-        <v>2187</v>
+        <v>2186</v>
       </c>
       <c r="EX12" s="4" t="s">
-        <v>289</v>
+        <v>717</v>
       </c>
       <c r="EY12" s="4"/>
       <c r="EZ12" s="4"/>
       <c r="FA12" s="4"/>
       <c r="FB12" s="4"/>
       <c r="FC12" s="4" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="FD12" s="4" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
     </row>
     <row r="13">
@@ -24958,20 +24967,20 @@
       <c r="EU13" s="4"/>
       <c r="EV13" s="4"/>
       <c r="EW13" s="4" t="s">
-        <v>2188</v>
+        <v>2187</v>
       </c>
       <c r="EX13" s="4" t="s">
-        <v>732</v>
+        <v>289</v>
       </c>
       <c r="EY13" s="4"/>
       <c r="EZ13" s="4"/>
       <c r="FA13" s="4"/>
       <c r="FB13" s="4"/>
       <c r="FC13" s="4" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="FD13" s="4" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="14">
@@ -25140,20 +25149,20 @@
       <c r="EU14" s="4"/>
       <c r="EV14" s="4"/>
       <c r="EW14" s="4" t="s">
-        <v>2189</v>
+        <v>2188</v>
       </c>
       <c r="EX14" s="4" t="s">
-        <v>2202</v>
+        <v>732</v>
       </c>
       <c r="EY14" s="4"/>
       <c r="EZ14" s="4"/>
       <c r="FA14" s="4"/>
       <c r="FB14" s="4"/>
       <c r="FC14" s="4" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="FD14" s="4" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="15">
@@ -25318,20 +25327,20 @@
       <c r="EU15" s="4"/>
       <c r="EV15" s="4"/>
       <c r="EW15" s="4" t="s">
-        <v>2190</v>
+        <v>2189</v>
       </c>
       <c r="EX15" s="4" t="s">
-        <v>2203</v>
+        <v>2204</v>
       </c>
       <c r="EY15" s="4"/>
       <c r="EZ15" s="4"/>
       <c r="FA15" s="4"/>
       <c r="FB15" s="4"/>
       <c r="FC15" s="4" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="FD15" s="4" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
     </row>
     <row r="16">
@@ -25496,20 +25505,20 @@
       <c r="EU16" s="4"/>
       <c r="EV16" s="4"/>
       <c r="EW16" s="4" t="s">
-        <v>2191</v>
+        <v>2190</v>
       </c>
       <c r="EX16" s="4" t="s">
-        <v>2204</v>
+        <v>2205</v>
       </c>
       <c r="EY16" s="4"/>
       <c r="EZ16" s="4"/>
       <c r="FA16" s="4"/>
       <c r="FB16" s="4"/>
       <c r="FC16" s="4" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="FD16" s="4" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
     </row>
     <row r="17">
@@ -25674,20 +25683,20 @@
       <c r="EU17" s="4"/>
       <c r="EV17" s="4"/>
       <c r="EW17" s="4" t="s">
-        <v>2192</v>
+        <v>2191</v>
       </c>
       <c r="EX17" s="4" t="s">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="EY17" s="4"/>
       <c r="EZ17" s="4"/>
       <c r="FA17" s="4"/>
       <c r="FB17" s="4"/>
       <c r="FC17" s="4" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="FD17" s="4" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="18">
@@ -25852,20 +25861,20 @@
       <c r="EU18" s="4"/>
       <c r="EV18" s="4"/>
       <c r="EW18" s="4" t="s">
-        <v>129</v>
+        <v>2192</v>
       </c>
       <c r="EX18" s="4" t="s">
-        <v>2206</v>
+        <v>2207</v>
       </c>
       <c r="EY18" s="4"/>
       <c r="EZ18" s="4"/>
       <c r="FA18" s="4"/>
       <c r="FB18" s="4"/>
       <c r="FC18" s="4" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="FD18" s="4" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="19">
@@ -26026,20 +26035,20 @@
       <c r="EU19" s="4"/>
       <c r="EV19" s="4"/>
       <c r="EW19" s="4" t="s">
-        <v>2193</v>
+        <v>129</v>
       </c>
       <c r="EX19" s="4" t="s">
-        <v>2207</v>
+        <v>2208</v>
       </c>
       <c r="EY19" s="4"/>
       <c r="EZ19" s="4"/>
       <c r="FA19" s="4"/>
       <c r="FB19" s="4"/>
       <c r="FC19" s="4" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="FD19" s="4" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="20">
@@ -26200,20 +26209,20 @@
       <c r="EU20" s="4"/>
       <c r="EV20" s="4"/>
       <c r="EW20" s="4" t="s">
-        <v>2194</v>
+        <v>2193</v>
       </c>
       <c r="EX20" s="4" t="s">
-        <v>2208</v>
+        <v>2209</v>
       </c>
       <c r="EY20" s="4"/>
       <c r="EZ20" s="4"/>
       <c r="FA20" s="4"/>
       <c r="FB20" s="4"/>
       <c r="FC20" s="4" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="FD20" s="4" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="21">
@@ -26373,17 +26382,21 @@
       <c r="ET21" s="4"/>
       <c r="EU21" s="4"/>
       <c r="EV21" s="4"/>
-      <c r="EW21" s="4"/>
-      <c r="EX21" s="4"/>
+      <c r="EW21" s="4" t="s">
+        <v>2194</v>
+      </c>
+      <c r="EX21" s="4" t="s">
+        <v>2210</v>
+      </c>
       <c r="EY21" s="4"/>
       <c r="EZ21" s="4"/>
       <c r="FA21" s="4"/>
       <c r="FB21" s="4"/>
       <c r="FC21" s="4" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="FD21" s="4" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="22">
@@ -26539,17 +26552,21 @@
       <c r="ET22" s="4"/>
       <c r="EU22" s="4"/>
       <c r="EV22" s="4"/>
-      <c r="EW22" s="4"/>
-      <c r="EX22" s="4"/>
+      <c r="EW22" s="4" t="s">
+        <v>2195</v>
+      </c>
+      <c r="EX22" s="4" t="s">
+        <v>2211</v>
+      </c>
       <c r="EY22" s="4"/>
       <c r="EZ22" s="4"/>
       <c r="FA22" s="4"/>
       <c r="FB22" s="4"/>
       <c r="FC22" s="4" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="FD22" s="4" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
     </row>
     <row r="23">
@@ -26712,10 +26729,10 @@
       <c r="FA23" s="4"/>
       <c r="FB23" s="4"/>
       <c r="FC23" s="4" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="FD23" s="4" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
     </row>
     <row r="24">
@@ -26878,10 +26895,10 @@
       <c r="FA24" s="4"/>
       <c r="FB24" s="4"/>
       <c r="FC24" s="4" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="FD24" s="4" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="25">
@@ -27044,10 +27061,10 @@
       <c r="FA25" s="4"/>
       <c r="FB25" s="4"/>
       <c r="FC25" s="4" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="FD25" s="4" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="26">
@@ -27210,10 +27227,10 @@
       <c r="FA26" s="4"/>
       <c r="FB26" s="4"/>
       <c r="FC26" s="4" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="FD26" s="4" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
     </row>
     <row r="27">
@@ -27379,7 +27396,7 @@
         <v>2189</v>
       </c>
       <c r="FD27" s="4" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="28">
@@ -27542,10 +27559,10 @@
       <c r="FA28" s="4"/>
       <c r="FB28" s="4"/>
       <c r="FC28" s="4" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="FD28" s="4" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="29">
@@ -27708,10 +27725,10 @@
       <c r="FA29" s="4"/>
       <c r="FB29" s="4"/>
       <c r="FC29" s="4" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="FD29" s="4" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="30">
@@ -27874,10 +27891,10 @@
       <c r="FA30" s="4"/>
       <c r="FB30" s="4"/>
       <c r="FC30" s="4" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="FD30" s="4" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="31">
@@ -28040,10 +28057,10 @@
       <c r="FA31" s="4"/>
       <c r="FB31" s="4"/>
       <c r="FC31" s="4" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="FD31" s="4" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="32">
@@ -28206,10 +28223,10 @@
       <c r="FA32" s="4"/>
       <c r="FB32" s="4"/>
       <c r="FC32" s="4" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="FD32" s="4" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="33">
@@ -28372,10 +28389,10 @@
       <c r="FA33" s="4"/>
       <c r="FB33" s="4"/>
       <c r="FC33" s="4" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="FD33" s="4" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
     </row>
     <row r="34">
@@ -28538,10 +28555,10 @@
       <c r="FA34" s="4"/>
       <c r="FB34" s="4"/>
       <c r="FC34" s="4" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="FD34" s="4" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
     </row>
     <row r="35">
@@ -28704,10 +28721,10 @@
       <c r="FA35" s="4"/>
       <c r="FB35" s="4"/>
       <c r="FC35" s="4" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="FD35" s="4" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
     </row>
     <row r="36">
@@ -28870,10 +28887,10 @@
       <c r="FA36" s="4"/>
       <c r="FB36" s="4"/>
       <c r="FC36" s="4" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="FD36" s="4" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
     </row>
     <row r="37">
@@ -29036,10 +29053,10 @@
       <c r="FA37" s="4"/>
       <c r="FB37" s="4"/>
       <c r="FC37" s="4" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="FD37" s="4" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="38">
@@ -29202,10 +29219,10 @@
       <c r="FA38" s="4"/>
       <c r="FB38" s="4"/>
       <c r="FC38" s="4" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="FD38" s="4" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="39">
@@ -29368,10 +29385,10 @@
       <c r="FA39" s="4"/>
       <c r="FB39" s="4"/>
       <c r="FC39" s="4" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="FD39" s="4" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
     </row>
   </sheetData>
@@ -29415,7 +29432,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>1</v>
@@ -29424,7 +29441,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>1</v>
@@ -29433,10 +29450,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="C5" s="3"/>
     </row>

</xml_diff>